<commit_message>
Allow manual catalog re-import after admin delete and harden bulk imports.
Mirror the pincode tombstone policy for categories, services, and sub-services so UI/import can restore deleted records while seeders stay blocked. Speed up workbook commits by suppressing per-row observer work, deferring post-sync, and fixing same-workbook preview linkage for sub-services.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/storage/imports/templates/services.xlsx
+++ b/storage/imports/templates/services.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="100">
   <si>
     <t>code</t>
   </si>
@@ -98,6 +98,18 @@
     <t>breadcrumb_title</t>
   </si>
   <si>
+    <t>physiotherapy</t>
+  </si>
+  <si>
+    <t>Physiotherapy at Home</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>public</t>
+  </si>
+  <si>
     <t>primary_category_code</t>
   </si>
   <si>
@@ -281,10 +293,31 @@
     <t>image_alt</t>
   </si>
   <si>
+    <t>SRV-PHYSIO-01</t>
+  </si>
+  <si>
+    <t>Expert physiotherapy in Bangalore (Arekere belt).</t>
+  </si>
+  <si>
+    <t>published</t>
+  </si>
+  <si>
     <t>parent_service_code</t>
   </si>
   <si>
     <t>sub_service_code</t>
+  </si>
+  <si>
+    <t>SUB-PHYSIO-NECK</t>
+  </si>
+  <si>
+    <t>Neck Pain Physiotherapy</t>
+  </si>
+  <si>
+    <t>SUB-PHYSIO-BACK</t>
+  </si>
+  <si>
+    <t>Back Pain Physiotherapy</t>
   </si>
 </sst>
 </file>
@@ -624,7 +657,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:26">
@@ -705,6 +738,20 @@
       </c>
       <c r="Z1" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -719,63 +766,63 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:CC1"/>
+  <dimension ref="A1:CC2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:81">
       <c r="A1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
       </c>
       <c r="G1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="J1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="K1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="L1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="M1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="N1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="O1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="P1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="Q1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="R1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="S1" t="s">
         <v>5</v>
@@ -784,7 +831,7 @@
         <v>6</v>
       </c>
       <c r="U1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="V1" t="s">
         <v>8</v>
@@ -817,13 +864,13 @@
         <v>20</v>
       </c>
       <c r="AF1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AG1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="AH1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="AI1" t="s">
         <v>25</v>
@@ -832,61 +879,61 @@
         <v>24</v>
       </c>
       <c r="AK1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="AL1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="AM1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="AN1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AO1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="AP1" t="s">
         <v>23</v>
       </c>
       <c r="AQ1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="AR1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="AS1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="AT1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="AU1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="AV1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="AW1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="AX1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="AY1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="AZ1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="BA1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="BB1" t="s">
         <v>7</v>
       </c>
       <c r="BC1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="BD1" t="s">
         <v>9</v>
@@ -898,73 +945,99 @@
         <v>11</v>
       </c>
       <c r="BG1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="BH1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="BI1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="BJ1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="BK1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="BL1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="BM1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="BN1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="BO1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="BP1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="BQ1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="BR1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="BS1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="BT1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="BU1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="BV1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="BW1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="BX1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="BY1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="BZ1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="CA1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="CB1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="CC1" t="s">
-        <v>86</v>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:81">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>92</v>
+      </c>
+      <c r="T2" t="s">
+        <v>28</v>
+      </c>
+      <c r="U2" t="s">
+        <v>93</v>
+      </c>
+      <c r="V2" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -979,21 +1052,21 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:X3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:24">
       <c r="A1" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -1005,7 +1078,7 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I1" t="s">
         <v>8</v>
@@ -1014,7 +1087,7 @@
         <v>7</v>
       </c>
       <c r="K1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="L1" t="s">
         <v>9</v>
@@ -1041,19 +1114,59 @@
         <v>23</v>
       </c>
       <c r="T1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="U1" t="s">
         <v>24</v>
       </c>
       <c r="V1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="W1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="X1" t="s">
-        <v>62</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24">
+      <c r="A2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" t="s">
+        <v>93</v>
+      </c>
+      <c r="I2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24">
+      <c r="A3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" t="s">
+        <v>93</v>
+      </c>
+      <c r="I3" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1073,37 +1186,37 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="I1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="J1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="K1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ship catalog parity, nested navigation, admin notifications, and updated import templates.
Align categories, services, and sub-services with shared master fields in Operations and services.xlsx; add nested Site Architect navigation with catalog auto-sync and drag controls; fan out admin notification bell UI; and harden public service/category presentation.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/storage/imports/templates/services.xlsx
+++ b/storage/imports/templates/services.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="103">
   <si>
     <t>code</t>
   </si>
@@ -32,6 +32,9 @@
     <t>description</t>
   </si>
   <si>
+    <t>short_summary</t>
+  </si>
+  <si>
     <t>parent_code</t>
   </si>
   <si>
@@ -44,6 +47,9 @@
     <t>is_featured</t>
   </si>
   <si>
+    <t>publish_status</t>
+  </si>
+  <si>
     <t>visibility</t>
   </si>
   <si>
@@ -56,6 +62,39 @@
     <t>show_on_contact</t>
   </si>
   <si>
+    <t>key_benefits</t>
+  </si>
+  <si>
+    <t>eligibility</t>
+  </si>
+  <si>
+    <t>process_steps</t>
+  </si>
+  <si>
+    <t>ai_summary</t>
+  </si>
+  <si>
+    <t>procedures</t>
+  </si>
+  <si>
+    <t>specialized_care</t>
+  </si>
+  <si>
+    <t>shifts</t>
+  </si>
+  <si>
+    <t>price_range</t>
+  </si>
+  <si>
+    <t>trust_signals</t>
+  </si>
+  <si>
+    <t>target_keywords</t>
+  </si>
+  <si>
+    <t>ai_keywords</t>
+  </si>
+  <si>
     <t>meta_title</t>
   </si>
   <si>
@@ -89,13 +128,43 @@
     <t>aeo_answer</t>
   </si>
   <si>
+    <t>h1</t>
+  </si>
+  <si>
+    <t>h2_lines</t>
+  </si>
+  <si>
+    <t>h3_lines</t>
+  </si>
+  <si>
+    <t>search_intent</t>
+  </si>
+  <si>
+    <t>ai_context</t>
+  </si>
+  <si>
+    <t>breadcrumb_title</t>
+  </si>
+  <si>
     <t>faq_pairs</t>
   </si>
   <si>
-    <t>h1</t>
-  </si>
-  <si>
-    <t>breadcrumb_title</t>
+    <t>schema_type</t>
+  </si>
+  <si>
+    <t>schema_json_override</t>
+  </si>
+  <si>
+    <t>featured_image_url</t>
+  </si>
+  <si>
+    <t>icon_url</t>
+  </si>
+  <si>
+    <t>gallery_image_urls</t>
+  </si>
+  <si>
+    <t>image_alt</t>
   </si>
   <si>
     <t>physiotherapy</t>
@@ -104,9 +173,15 @@
     <t>Physiotherapy at Home</t>
   </si>
   <si>
+    <t>Licensed physiotherapy delivered at home across Bangalore.</t>
+  </si>
+  <si>
     <t>TRUE</t>
   </si>
   <si>
+    <t>published</t>
+  </si>
+  <si>
     <t>public</t>
   </si>
   <si>
@@ -122,18 +197,6 @@
     <t>title</t>
   </si>
   <si>
-    <t>short_summary</t>
-  </si>
-  <si>
-    <t>key_benefits</t>
-  </si>
-  <si>
-    <t>eligibility</t>
-  </si>
-  <si>
-    <t>process_steps</t>
-  </si>
-  <si>
     <t>preparation</t>
   </si>
   <si>
@@ -146,24 +209,12 @@
     <t>deliverables</t>
   </si>
   <si>
-    <t>trust_signals</t>
-  </si>
-  <si>
-    <t>procedures</t>
-  </si>
-  <si>
-    <t>shifts</t>
-  </si>
-  <si>
     <t>coverage_notes</t>
   </si>
   <si>
     <t>emergency_coverage_notes</t>
   </si>
   <si>
-    <t>publish_status</t>
-  </si>
-  <si>
     <t>twitter_title</t>
   </si>
   <si>
@@ -173,12 +224,6 @@
     <t>twitter_image</t>
   </si>
   <si>
-    <t>h2_lines</t>
-  </si>
-  <si>
-    <t>h3_lines</t>
-  </si>
-  <si>
     <t>h4_lines</t>
   </si>
   <si>
@@ -188,18 +233,9 @@
     <t>h6_lines</t>
   </si>
   <si>
-    <t>ai_summary</t>
-  </si>
-  <si>
     <t>ai_recommendation_summary</t>
   </si>
   <si>
-    <t>target_keywords</t>
-  </si>
-  <si>
-    <t>ai_keywords</t>
-  </si>
-  <si>
     <t>voice_search_queries</t>
   </si>
   <si>
@@ -209,18 +245,6 @@
     <t>entity_references</t>
   </si>
   <si>
-    <t>search_intent</t>
-  </si>
-  <si>
-    <t>ai_context</t>
-  </si>
-  <si>
-    <t>schema_type</t>
-  </si>
-  <si>
-    <t>schema_json_override</t>
-  </si>
-  <si>
     <t>is_top_rated</t>
   </si>
   <si>
@@ -275,31 +299,16 @@
     <t>location_meta_description_template</t>
   </si>
   <si>
-    <t>featured_image_url</t>
-  </si>
-  <si>
     <t>banner_image_url</t>
   </si>
   <si>
-    <t>icon_url</t>
-  </si>
-  <si>
-    <t>gallery_image_urls</t>
-  </si>
-  <si>
     <t>video_url</t>
   </si>
   <si>
-    <t>image_alt</t>
-  </si>
-  <si>
     <t>SRV-PHYSIO-01</t>
   </si>
   <si>
     <t>Expert physiotherapy in Bangalore (Arekere belt).</t>
-  </si>
-  <si>
-    <t>published</t>
   </si>
   <si>
     <t>parent_service_code</t>
@@ -657,10 +666,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AW2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:26">
+    <row r="1" spans="1:49">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -739,19 +748,94 @@
       <c r="Z1" t="s">
         <v>25</v>
       </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>48</v>
+      </c>
     </row>
-    <row r="2" spans="1:26">
+    <row r="2" spans="1:49">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I2" t="s">
-        <v>29</v>
+        <v>50</v>
+      </c>
+      <c r="E2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K2" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -766,278 +850,281 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:CC2"/>
+  <dimension ref="A1:CD2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:81">
+    <row r="1" spans="1:82">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
       </c>
       <c r="G1" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="H1" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="I1" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="J1" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="K1" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="L1" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="M1" t="s">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="N1" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="O1" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="P1" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="Q1" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="R1" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="S1" t="s">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="T1" t="s">
         <v>6</v>
       </c>
       <c r="U1" t="s">
+        <v>7</v>
+      </c>
+      <c r="V1" t="s">
+        <v>9</v>
+      </c>
+      <c r="W1" t="s">
+        <v>10</v>
+      </c>
+      <c r="X1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>70</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>73</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>74</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>40</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>43</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>8</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>75</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>11</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>12</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>13</v>
+      </c>
+      <c r="BH1" t="s">
+        <v>76</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>77</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>78</v>
+      </c>
+      <c r="BK1" t="s">
+        <v>79</v>
+      </c>
+      <c r="BL1" t="s">
+        <v>80</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>81</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>82</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>83</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>84</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>85</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>86</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>87</v>
+      </c>
+      <c r="BT1" t="s">
+        <v>88</v>
+      </c>
+      <c r="BU1" t="s">
+        <v>89</v>
+      </c>
+      <c r="BV1" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW1" t="s">
+        <v>91</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>92</v>
+      </c>
+      <c r="BY1" t="s">
+        <v>45</v>
+      </c>
+      <c r="BZ1" t="s">
+        <v>93</v>
+      </c>
+      <c r="CA1" t="s">
+        <v>46</v>
+      </c>
+      <c r="CB1" t="s">
         <v>47</v>
       </c>
-      <c r="V1" t="s">
-        <v>8</v>
-      </c>
-      <c r="W1" t="s">
-        <v>12</v>
-      </c>
-      <c r="X1" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>15</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>16</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>17</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>18</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>19</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>20</v>
-      </c>
-      <c r="AF1" t="s">
+      <c r="CC1" t="s">
+        <v>94</v>
+      </c>
+      <c r="CD1" t="s">
         <v>48</v>
       </c>
-      <c r="AG1" t="s">
+    </row>
+    <row r="2" spans="1:82">
+      <c r="A2" t="s">
         <v>49</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="B2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" t="s">
         <v>50</v>
       </c>
-      <c r="AI1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AL1" t="s">
+      <c r="E2" t="s">
+        <v>96</v>
+      </c>
+      <c r="U2" t="s">
         <v>52</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="V2" t="s">
         <v>53</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="W2" t="s">
         <v>54</v>
-      </c>
-      <c r="AO1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>23</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AR1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AS1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AT1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AU1" t="s">
-        <v>60</v>
-      </c>
-      <c r="AV1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AW1" t="s">
-        <v>62</v>
-      </c>
-      <c r="AX1" t="s">
-        <v>63</v>
-      </c>
-      <c r="AY1" t="s">
-        <v>64</v>
-      </c>
-      <c r="AZ1" t="s">
-        <v>65</v>
-      </c>
-      <c r="BA1" t="s">
-        <v>66</v>
-      </c>
-      <c r="BB1" t="s">
-        <v>7</v>
-      </c>
-      <c r="BC1" t="s">
-        <v>67</v>
-      </c>
-      <c r="BD1" t="s">
-        <v>9</v>
-      </c>
-      <c r="BE1" t="s">
-        <v>10</v>
-      </c>
-      <c r="BF1" t="s">
-        <v>11</v>
-      </c>
-      <c r="BG1" t="s">
-        <v>68</v>
-      </c>
-      <c r="BH1" t="s">
-        <v>69</v>
-      </c>
-      <c r="BI1" t="s">
-        <v>70</v>
-      </c>
-      <c r="BJ1" t="s">
-        <v>71</v>
-      </c>
-      <c r="BK1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BL1" t="s">
-        <v>73</v>
-      </c>
-      <c r="BM1" t="s">
-        <v>74</v>
-      </c>
-      <c r="BN1" t="s">
-        <v>75</v>
-      </c>
-      <c r="BO1" t="s">
-        <v>76</v>
-      </c>
-      <c r="BP1" t="s">
-        <v>77</v>
-      </c>
-      <c r="BQ1" t="s">
-        <v>78</v>
-      </c>
-      <c r="BR1" t="s">
-        <v>79</v>
-      </c>
-      <c r="BS1" t="s">
-        <v>80</v>
-      </c>
-      <c r="BT1" t="s">
-        <v>81</v>
-      </c>
-      <c r="BU1" t="s">
-        <v>82</v>
-      </c>
-      <c r="BV1" t="s">
-        <v>83</v>
-      </c>
-      <c r="BW1" t="s">
-        <v>84</v>
-      </c>
-      <c r="BX1" t="s">
-        <v>85</v>
-      </c>
-      <c r="BY1" t="s">
-        <v>86</v>
-      </c>
-      <c r="BZ1" t="s">
-        <v>87</v>
-      </c>
-      <c r="CA1" t="s">
-        <v>88</v>
-      </c>
-      <c r="CB1" t="s">
-        <v>89</v>
-      </c>
-      <c r="CC1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="2" spans="1:81">
-      <c r="A2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" t="s">
-        <v>92</v>
-      </c>
-      <c r="T2" t="s">
-        <v>28</v>
-      </c>
-      <c r="U2" t="s">
-        <v>93</v>
-      </c>
-      <c r="V2" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1052,121 +1139,187 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:AT3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:46">
       <c r="A1" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C1" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="D1" t="s">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N1" t="s">
+        <v>22</v>
+      </c>
+      <c r="O1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="R1" t="s">
+        <v>7</v>
+      </c>
+      <c r="S1" t="s">
+        <v>9</v>
+      </c>
+      <c r="T1" t="s">
+        <v>10</v>
+      </c>
+      <c r="U1" t="s">
+        <v>8</v>
+      </c>
+      <c r="V1" t="s">
+        <v>75</v>
+      </c>
+      <c r="W1" t="s">
+        <v>11</v>
+      </c>
+      <c r="X1" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AS1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" t="s">
-        <v>67</v>
-      </c>
-      <c r="L1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" t="s">
-        <v>12</v>
-      </c>
-      <c r="P1" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>14</v>
-      </c>
-      <c r="R1" t="s">
-        <v>15</v>
-      </c>
-      <c r="S1" t="s">
-        <v>23</v>
-      </c>
-      <c r="T1" t="s">
-        <v>56</v>
-      </c>
-      <c r="U1" t="s">
-        <v>24</v>
-      </c>
-      <c r="V1" t="s">
-        <v>51</v>
-      </c>
-      <c r="W1" t="s">
+      <c r="AT1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:46">
+      <c r="A2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" t="s">
+        <v>100</v>
+      </c>
+      <c r="R2" t="s">
         <v>52</v>
       </c>
-      <c r="X1" t="s">
-        <v>66</v>
+      <c r="S2" t="s">
+        <v>53</v>
+      </c>
+      <c r="T2" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:24">
-      <c r="A2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" t="s">
-        <v>97</v>
-      </c>
-      <c r="G2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H2" t="s">
-        <v>93</v>
-      </c>
-      <c r="I2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:46">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H3" t="s">
-        <v>93</v>
-      </c>
-      <c r="I3" t="s">
-        <v>29</v>
+        <v>102</v>
+      </c>
+      <c r="R3" t="s">
+        <v>52</v>
+      </c>
+      <c r="S3" t="s">
+        <v>53</v>
+      </c>
+      <c r="T3" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1186,37 +1339,37 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="C1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="D1" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="E1" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="G1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="H1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="I1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="J1" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="K1" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>